<commit_message>
Final clean and Git Push
</commit_message>
<xml_diff>
--- a/BDDCucumberFramework/src/main/java/Testdata/New Customer creation sheet.xlsx
+++ b/BDDCucumberFramework/src/main/java/Testdata/New Customer creation sheet.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>URL</t>
   </si>
@@ -35,6 +35,24 @@
   </si>
   <si>
     <t>184776</t>
+  </si>
+  <si>
+    <t>27668</t>
+  </si>
+  <si>
+    <t>185173</t>
+  </si>
+  <si>
+    <t>19614</t>
+  </si>
+  <si>
+    <t>185177</t>
+  </si>
+  <si>
+    <t>27924</t>
+  </si>
+  <si>
+    <t>185178</t>
   </si>
 </sst>
 </file>
@@ -407,10 +425,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>